<commit_message>
fix(rh): feuille de temps — blocs résiduels du modèle supprimés, date longue
Le gabarit conservait les blocs semaines 2-7 du modèle Microsoft
(lignes 20-73, données décembre 2025 et bandeaux gris) sous le bloc
rempli. Gabarit reconstruit : bloc unique + sa ligne « Nombre total
d'heures » (formules conservées). Format de date aligné sur le modèle
(date longue système : « lundi 1 décembre 2025 »).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XA7hsDjgUhFae2VXUBXjih
</commit_message>
<xml_diff>
--- a/feuille_temps_template.xlsx
+++ b/feuille_temps_template.xlsx
@@ -649,7 +649,7 @@
     <xf numFmtId="0" fontId="1" fillId="33" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="34" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -842,18 +842,6 @@
     </xf>
     <xf numFmtId="165" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="25" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="55">
@@ -15120,7 +15108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:K73"/>
+  <dimension ref="B1:K19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col width="2.625" customWidth="1" style="2" min="1" max="1"/>
@@ -15384,11 +15372,7 @@
       </c>
       <c r="I14" s="15" t="n"/>
       <c r="J14" s="15" t="n"/>
-      <c r="K14" s="15" t="inlineStr">
-        <is>
-          <t>(+) 1h</t>
-        </is>
-      </c>
+      <c r="K14" s="15" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1" s="58">
       <c r="B15" s="61" t="n"/>
@@ -15495,1255 +15479,54 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="14.25" customHeight="1" s="58">
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Jour</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Arrivée</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Départ</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Arrivée </t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Départ </t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>Heures normales</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>Heures supplémentaires</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>Heures d’arrêt maladie</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>Heures de congés</t>
-        </is>
-      </c>
-      <c r="K20" s="10" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1" s="58">
-      <c r="B21" s="61" t="n">
-        <v>45992</v>
-      </c>
-      <c r="C21" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D21" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E21" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F21" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G21" s="14">
-        <f>(D21-C21)+(F21-E21)</f>
-        <v/>
-      </c>
-      <c r="H21" s="15">
-        <f>(G21-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I21" s="15" t="n"/>
-      <c r="J21" s="15" t="n"/>
-      <c r="K21" s="15" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1" s="58">
-      <c r="B22" s="61" t="n">
-        <v>45993</v>
-      </c>
-      <c r="C22" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D22" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E22" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G22" s="14">
-        <f>(D22-C22)+(F22-E22)</f>
-        <v/>
-      </c>
-      <c r="H22" s="15">
-        <f>(G22-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I22" s="15" t="n"/>
-      <c r="J22" s="15" t="n"/>
-      <c r="K22" s="15" t="n"/>
-    </row>
-    <row r="23" ht="30" customHeight="1" s="58">
-      <c r="B23" s="61" t="n">
-        <v>45994</v>
-      </c>
-      <c r="C23" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D23" s="13" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="E23" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F23" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G23" s="14">
-        <f>(D23-C23)+(F23-E23)</f>
-        <v/>
-      </c>
-      <c r="H23" s="16">
-        <f>(G23-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I23" s="15" t="n"/>
-      <c r="J23" s="15" t="n"/>
-      <c r="K23" s="15" t="inlineStr">
-        <is>
-          <t>(+) 1h</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1" s="58">
-      <c r="B24" s="61" t="n">
-        <v>45995</v>
-      </c>
-      <c r="C24" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D24" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E24" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F24" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G24" s="14">
-        <f>(D24-C24)+(F24-E24)</f>
-        <v/>
-      </c>
-      <c r="H24" s="15">
-        <f>(G24-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="15" t="n"/>
-      <c r="K24" s="15" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1" s="58">
-      <c r="B25" s="61" t="n">
-        <v>45996</v>
-      </c>
-      <c r="C25" s="13" t="n">
-        <v>0.2916666666666667</v>
-      </c>
-      <c r="D25" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="13" t="n"/>
-      <c r="G25" s="14">
-        <f>(D25-C25)+(F25-E25)</f>
-        <v/>
-      </c>
-      <c r="H25" s="15">
-        <f>(G25-F2)*24</f>
-        <v/>
-      </c>
-      <c r="I25" s="15" t="n"/>
-      <c r="J25" s="15" t="n"/>
-      <c r="K25" s="15" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1" s="58">
-      <c r="B26" s="61" t="n">
-        <v>45997</v>
-      </c>
-      <c r="C26" s="13" t="n"/>
-      <c r="D26" s="13" t="n"/>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="13" t="n"/>
-      <c r="G26" s="17">
-        <f>(D26-C26)+(F26-E26)</f>
-        <v/>
-      </c>
-      <c r="H26" s="15">
-        <f>ABS((G26-E6)*24)</f>
-        <v/>
-      </c>
-      <c r="I26" s="15" t="n"/>
-      <c r="J26" s="15" t="n"/>
-      <c r="K26" s="15">
-        <f>IFERROR(SUM(G26:J26), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1" s="58">
-      <c r="B27" s="61" t="n">
-        <v>45998</v>
-      </c>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="13" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="17">
-        <f>(D27-C27)+(F27-E27)</f>
-        <v/>
-      </c>
-      <c r="H27" s="15">
-        <f>ABS((G27-E7)*24)</f>
-        <v/>
-      </c>
-      <c r="I27" s="15" t="n"/>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="15">
-        <f>IFERROR(SUM(G27:J27), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1" s="58">
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>Nombre total d’heures</t>
-        </is>
-      </c>
-      <c r="G28" s="19">
-        <f>SUM(G21:G27)*24</f>
-        <v/>
-      </c>
-      <c r="H28" s="20">
-        <f>SUM(H21:H27)</f>
-        <v/>
-      </c>
-      <c r="I28" s="19">
-        <f>SUM(I21:I27)</f>
-        <v/>
-      </c>
-      <c r="J28" s="19">
-        <f>SUM(J21:J27)</f>
-        <v/>
-      </c>
-      <c r="K28" s="21">
-        <f>SUM(TimeSheet3[Total])</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="14.25" customHeight="1" s="58">
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Jour</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Arrivée</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>Départ</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Arrivée </t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Départ </t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="inlineStr">
-        <is>
-          <t>Heures normales</t>
-        </is>
-      </c>
-      <c r="H29" s="11" t="inlineStr">
-        <is>
-          <t>Heures supplémentaires</t>
-        </is>
-      </c>
-      <c r="I29" s="11" t="inlineStr">
-        <is>
-          <t>Heures d’arrêt maladie</t>
-        </is>
-      </c>
-      <c r="J29" s="10" t="inlineStr">
-        <is>
-          <t>Heures de congés</t>
-        </is>
-      </c>
-      <c r="K29" s="10" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1" s="58">
-      <c r="B30" s="61" t="n">
-        <v>45999</v>
-      </c>
-      <c r="C30" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D30" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E30" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G30" s="14">
-        <f>(D30-C30)+(F30-E30)</f>
-        <v/>
-      </c>
-      <c r="H30" s="15">
-        <f>(G30-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I30" s="15" t="n"/>
-      <c r="J30" s="15" t="n"/>
-      <c r="K30" s="15" t="n"/>
-    </row>
-    <row r="31" ht="30" customHeight="1" s="58">
-      <c r="B31" s="61" t="n">
-        <v>46000</v>
-      </c>
-      <c r="C31" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D31" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E31" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F31" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G31" s="14">
-        <f>(D31-C31)+(F31-E31)</f>
-        <v/>
-      </c>
-      <c r="H31" s="15">
-        <f>(G31-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I31" s="15" t="n"/>
-      <c r="J31" s="15" t="n"/>
-      <c r="K31" s="15" t="n"/>
-    </row>
-    <row r="32" ht="30" customHeight="1" s="58">
-      <c r="B32" s="61" t="n">
-        <v>46001</v>
-      </c>
-      <c r="C32" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D32" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E32" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F32" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G32" s="14">
-        <f>(D32-C32)+(F32-E32)</f>
-        <v/>
-      </c>
-      <c r="H32" s="15">
-        <f>(G32-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I32" s="15" t="n"/>
-      <c r="J32" s="15" t="n"/>
-      <c r="K32" s="15" t="n"/>
-    </row>
-    <row r="33" ht="30" customHeight="1" s="58">
-      <c r="B33" s="61" t="n">
-        <v>46002</v>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D33" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E33" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F33" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G33" s="14">
-        <f>(D33-C33)+(F33-E33)</f>
-        <v/>
-      </c>
-      <c r="H33" s="15">
-        <f>(G33-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I33" s="15" t="n"/>
-      <c r="J33" s="15" t="n"/>
-      <c r="K33" s="15" t="n"/>
-    </row>
-    <row r="34" ht="30" customHeight="1" s="58">
-      <c r="B34" s="61" t="n">
-        <v>46003</v>
-      </c>
-      <c r="C34" s="13" t="n">
-        <v>0.2916666666666667</v>
-      </c>
-      <c r="D34" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n"/>
-      <c r="G34" s="14">
-        <f>(D34-C34)+(F34-E34)</f>
-        <v/>
-      </c>
-      <c r="H34" s="15">
-        <f>(G34-F2)*24</f>
-        <v/>
-      </c>
-      <c r="I34" s="15" t="n"/>
-      <c r="J34" s="15" t="n"/>
-      <c r="K34" s="15" t="n"/>
-    </row>
-    <row r="35" ht="30" customHeight="1" s="58">
-      <c r="B35" s="61" t="n">
-        <v>46004</v>
-      </c>
-      <c r="C35" s="13" t="n"/>
-      <c r="D35" s="13" t="n"/>
-      <c r="E35" s="13" t="n"/>
-      <c r="F35" s="13" t="n"/>
-      <c r="G35" s="17">
-        <f>(D35-C35)+(F35-E35)</f>
-        <v/>
-      </c>
-      <c r="H35" s="15" t="n"/>
-      <c r="I35" s="15" t="n"/>
-      <c r="J35" s="15" t="n"/>
-      <c r="K35" s="15">
-        <f>IFERROR(SUM(G35:J35), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1" s="58">
-      <c r="B36" s="61" t="n">
-        <v>46005</v>
-      </c>
-      <c r="C36" s="13" t="n"/>
-      <c r="D36" s="13" t="n"/>
-      <c r="E36" s="13" t="n"/>
-      <c r="F36" s="13" t="n"/>
-      <c r="G36" s="17">
-        <f>(D36-C36)+(F36-E36)</f>
-        <v/>
-      </c>
-      <c r="H36" s="15">
-        <f>IFERROR(IF(((D36-C36)+(F36-E36))*24&gt;8,((D36-C36)+(F36-E36))*24-8,0), "")</f>
-        <v/>
-      </c>
-      <c r="I36" s="15" t="n"/>
-      <c r="J36" s="15" t="n"/>
-      <c r="K36" s="15">
-        <f>IFERROR(SUM(G36:J36), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1" s="58">
-      <c r="F37" s="18" t="inlineStr">
-        <is>
-          <t>Nombre total d’heures</t>
-        </is>
-      </c>
-      <c r="G37" s="19">
-        <f>SUM(G30:G36)*24</f>
-        <v/>
-      </c>
-      <c r="H37" s="20">
-        <f>SUM(H30:H36)</f>
-        <v/>
-      </c>
-      <c r="I37" s="19">
-        <f>SUM(I30:I36)</f>
-        <v/>
-      </c>
-      <c r="J37" s="19">
-        <f>SUM(J30:J36)</f>
-        <v/>
-      </c>
-      <c r="K37" s="21">
-        <f>SUM(TimeSheet34[Total])</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="14.25" customHeight="1" s="58">
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Jour</t>
-        </is>
-      </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>Arrivée</t>
-        </is>
-      </c>
-      <c r="D38" s="10" t="inlineStr">
-        <is>
-          <t>Départ</t>
-        </is>
-      </c>
-      <c r="E38" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Arrivée </t>
-        </is>
-      </c>
-      <c r="F38" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Départ </t>
-        </is>
-      </c>
-      <c r="G38" s="11" t="inlineStr">
-        <is>
-          <t>Heures normales</t>
-        </is>
-      </c>
-      <c r="H38" s="11" t="inlineStr">
-        <is>
-          <t>Heures supplémentaires</t>
-        </is>
-      </c>
-      <c r="I38" s="11" t="inlineStr">
-        <is>
-          <t>Heures d’arrêt maladie</t>
-        </is>
-      </c>
-      <c r="J38" s="10" t="inlineStr">
-        <is>
-          <t>Heures de congés</t>
-        </is>
-      </c>
-      <c r="K38" s="10" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1" s="58">
-      <c r="B39" s="61" t="n">
-        <v>46006</v>
-      </c>
-      <c r="C39" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D39" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E39" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F39" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G39" s="14">
-        <f>(D39-C39)+(F39-E39)</f>
-        <v/>
-      </c>
-      <c r="H39" s="15">
-        <f>(G39-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I39" s="15" t="n"/>
-      <c r="J39" s="15" t="n"/>
-      <c r="K39" s="15" t="n"/>
-    </row>
-    <row r="40" ht="30" customHeight="1" s="58">
-      <c r="B40" s="61" t="n">
-        <v>46007</v>
-      </c>
-      <c r="C40" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D40" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E40" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F40" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G40" s="14">
-        <f>(D40-C40)+(F40-E40)</f>
-        <v/>
-      </c>
-      <c r="H40" s="15">
-        <f>(G40-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I40" s="15" t="n"/>
-      <c r="J40" s="15" t="n"/>
-      <c r="K40" s="15" t="n"/>
-    </row>
-    <row r="41" ht="30" customHeight="1" s="58">
-      <c r="B41" s="61" t="n">
-        <v>46008</v>
-      </c>
-      <c r="C41" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D41" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E41" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F41" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G41" s="14">
-        <f>(D41-C41)+(F41-E41)</f>
-        <v/>
-      </c>
-      <c r="H41" s="15">
-        <f>(G41-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I41" s="15" t="n"/>
-      <c r="J41" s="15" t="n"/>
-      <c r="K41" s="15" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1" s="58">
-      <c r="B42" s="61" t="n">
-        <v>46009</v>
-      </c>
-      <c r="C42" s="13" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D42" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E42" s="13" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="F42" s="13" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="G42" s="14">
-        <f>(D42-C42)+(F42-E42)</f>
-        <v/>
-      </c>
-      <c r="H42" s="15">
-        <f>(G42-E2)*24</f>
-        <v/>
-      </c>
-      <c r="I42" s="15" t="n"/>
-      <c r="J42" s="15" t="n"/>
-      <c r="K42" s="15" t="n"/>
-    </row>
-    <row r="43" ht="30" customHeight="1" s="58">
-      <c r="B43" s="61" t="n">
-        <v>46010</v>
-      </c>
-      <c r="C43" s="13" t="n">
-        <v>0.2916666666666667</v>
-      </c>
-      <c r="D43" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E43" s="13" t="n"/>
-      <c r="F43" s="13" t="n"/>
-      <c r="G43" s="14">
-        <f>(D43-C43)+(F43-E43)</f>
-        <v/>
-      </c>
-      <c r="H43" s="15">
-        <f>(G43-F2)*24</f>
-        <v/>
-      </c>
-      <c r="I43" s="15" t="n"/>
-      <c r="J43" s="15" t="n"/>
-      <c r="K43" s="15" t="n"/>
-    </row>
-    <row r="44" ht="30" customHeight="1" s="58">
-      <c r="B44" s="61" t="n">
-        <v>46011</v>
-      </c>
-      <c r="C44" s="13" t="n"/>
-      <c r="D44" s="13" t="n"/>
-      <c r="E44" s="13" t="n"/>
-      <c r="F44" s="13" t="n"/>
-      <c r="G44" s="17">
-        <f>(D44-C44)+(F44-E44)</f>
-        <v/>
-      </c>
-      <c r="H44" s="15">
-        <f>(G44-E6)*24</f>
-        <v/>
-      </c>
-      <c r="I44" s="15" t="n"/>
-      <c r="J44" s="15" t="n"/>
-      <c r="K44" s="15" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1" s="58">
-      <c r="B45" s="61" t="n">
-        <v>46012</v>
-      </c>
-      <c r="C45" s="13" t="n"/>
-      <c r="D45" s="13" t="n"/>
-      <c r="E45" s="13" t="n"/>
-      <c r="F45" s="13" t="n"/>
-      <c r="G45" s="17">
-        <f>(D45-C45)+(F45-E45)</f>
-        <v/>
-      </c>
-      <c r="H45" s="15">
-        <f>(G45-E7)*24</f>
-        <v/>
-      </c>
-      <c r="I45" s="15" t="n"/>
-      <c r="J45" s="15" t="n"/>
-      <c r="K45" s="15">
-        <f>IFERROR(SUM(G45:J45), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="30" customHeight="1" s="58">
-      <c r="F46" s="18" t="inlineStr">
-        <is>
-          <t>Nombre total d’heures</t>
-        </is>
-      </c>
-      <c r="G46" s="19">
-        <f>SUM(G39:G45)*24</f>
-        <v/>
-      </c>
-      <c r="H46" s="19" t="n"/>
-      <c r="I46" s="19">
-        <f>SUM(I39:I45)</f>
-        <v/>
-      </c>
-      <c r="J46" s="19">
-        <f>SUM(J39:J45)</f>
-        <v/>
-      </c>
-      <c r="K46" s="21">
-        <f>SUM(TimeSheet35[Total])</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" hidden="1" ht="14.25" customHeight="1" s="58">
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>Jour</t>
-        </is>
-      </c>
-      <c r="C47" s="10" t="inlineStr">
-        <is>
-          <t>Arrivée</t>
-        </is>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>Départ</t>
-        </is>
-      </c>
-      <c r="E47" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Arrivée </t>
-        </is>
-      </c>
-      <c r="F47" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Départ </t>
-        </is>
-      </c>
-      <c r="G47" s="11" t="inlineStr">
-        <is>
-          <t>Heures normales</t>
-        </is>
-      </c>
-      <c r="H47" s="11" t="inlineStr">
-        <is>
-          <t>Colonne1</t>
-        </is>
-      </c>
-      <c r="I47" s="11" t="inlineStr">
-        <is>
-          <t>Heures d’arrêt maladie</t>
-        </is>
-      </c>
-      <c r="J47" s="10" t="inlineStr">
-        <is>
-          <t>Heures de congés</t>
-        </is>
-      </c>
-      <c r="K47" s="10" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B48" s="61" t="n">
-        <v>46013</v>
-      </c>
-      <c r="C48" s="13" t="n"/>
-      <c r="D48" s="13" t="n"/>
-      <c r="E48" s="13" t="n"/>
-      <c r="F48" s="13" t="n"/>
-      <c r="G48" s="17" t="n"/>
-      <c r="H48" s="15" t="n"/>
-      <c r="I48" s="15" t="n"/>
-      <c r="J48" s="15" t="n"/>
-      <c r="K48" s="15">
-        <f>IFERROR(SUM(G48:J48), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B49" s="61" t="n">
-        <v>46014</v>
-      </c>
-      <c r="C49" s="13" t="n"/>
-      <c r="D49" s="13" t="n"/>
-      <c r="E49" s="13" t="n"/>
-      <c r="F49" s="13" t="n"/>
-      <c r="G49" s="17">
-        <f>IFERROR(IF((((D49-C49)+(F49-E49))*24)&gt;8,8,((D49-C49)+(F49-E49))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H49" s="15" t="n"/>
-      <c r="I49" s="15" t="n"/>
-      <c r="J49" s="15" t="n"/>
-      <c r="K49" s="15">
-        <f>IFERROR(SUM(G49:J49), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B50" s="61" t="n">
-        <v>46015</v>
-      </c>
-      <c r="C50" s="13" t="n"/>
-      <c r="D50" s="13" t="n"/>
-      <c r="E50" s="13" t="n"/>
-      <c r="F50" s="13" t="n"/>
-      <c r="G50" s="17">
-        <f>IFERROR(IF((((D50-C50)+(F50-E50))*24)&gt;8,8,((D50-C50)+(F50-E50))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H50" s="15" t="n"/>
-      <c r="I50" s="15" t="n"/>
-      <c r="J50" s="15" t="n"/>
-      <c r="K50" s="15">
-        <f>IFERROR(SUM(G50:J50), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B51" s="61" t="n">
-        <v>46016</v>
-      </c>
-      <c r="C51" s="13" t="n"/>
-      <c r="D51" s="13" t="n"/>
-      <c r="E51" s="13" t="n"/>
-      <c r="F51" s="13" t="n"/>
-      <c r="G51" s="17">
-        <f>IFERROR(IF((((D51-C51)+(F51-E51))*24)&gt;8,8,((D51-C51)+(F51-E51))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H51" s="15" t="n"/>
-      <c r="I51" s="15" t="n"/>
-      <c r="J51" s="15" t="n"/>
-      <c r="K51" s="15">
-        <f>IFERROR(SUM(G51:J51), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B52" s="61" t="n">
-        <v>46017</v>
-      </c>
-      <c r="C52" s="13" t="n"/>
-      <c r="D52" s="13" t="n"/>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="13" t="n"/>
-      <c r="G52" s="17">
-        <f>IFERROR(IF((((D52-C52)+(F52-E52))*24)&gt;8,8,((D52-C52)+(F52-E52))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H52" s="15" t="n"/>
-      <c r="I52" s="15" t="n"/>
-      <c r="J52" s="15" t="n"/>
-      <c r="K52" s="15">
-        <f>IFERROR(SUM(G52:J52), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B53" s="61" t="n">
-        <v>46018</v>
-      </c>
-      <c r="C53" s="13" t="n"/>
-      <c r="D53" s="13" t="n"/>
-      <c r="E53" s="13" t="n"/>
-      <c r="F53" s="13" t="n"/>
-      <c r="G53" s="17">
-        <f>IFERROR(IF((((D53-C53)+(F53-E53))*24)&gt;8,8,((D53-C53)+(F53-E53))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H53" s="15" t="n"/>
-      <c r="I53" s="15" t="n"/>
-      <c r="J53" s="15" t="n"/>
-      <c r="K53" s="15">
-        <f>IFERROR(SUM(G53:J53), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B54" s="61" t="n">
-        <v>46019</v>
-      </c>
-      <c r="C54" s="13" t="n"/>
-      <c r="D54" s="13" t="n"/>
-      <c r="E54" s="13" t="n"/>
-      <c r="F54" s="13" t="n"/>
-      <c r="G54" s="17">
-        <f>IFERROR(IF((((D54-C54)+(F54-E54))*24)&gt;8,8,((D54-C54)+(F54-E54))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H54" s="15" t="n"/>
-      <c r="I54" s="15" t="n"/>
-      <c r="J54" s="15" t="n"/>
-      <c r="K54" s="15">
-        <f>IFERROR(SUM(G54:J54), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="F55" s="18" t="inlineStr">
-        <is>
-          <t>Nombre total d’heures</t>
-        </is>
-      </c>
-      <c r="G55" s="19">
-        <f>SUM(G48:G54)</f>
-        <v/>
-      </c>
-      <c r="H55" s="19" t="n"/>
-      <c r="I55" s="19">
-        <f>SUM(I48:I54)</f>
-        <v/>
-      </c>
-      <c r="J55" s="19">
-        <f>SUM(J48:J54)</f>
-        <v/>
-      </c>
-      <c r="K55" s="21">
-        <f>SUM(TimeSheet36[Total])</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" hidden="1" ht="14.25" customHeight="1" s="58">
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t>Jour</t>
-        </is>
-      </c>
-      <c r="C56" s="10" t="inlineStr">
-        <is>
-          <t>Arrivée</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="inlineStr">
-        <is>
-          <t>Départ</t>
-        </is>
-      </c>
-      <c r="E56" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Arrivée </t>
-        </is>
-      </c>
-      <c r="F56" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Départ </t>
-        </is>
-      </c>
-      <c r="G56" s="11" t="inlineStr">
-        <is>
-          <t>Heures normales</t>
-        </is>
-      </c>
-      <c r="H56" s="11" t="inlineStr">
-        <is>
-          <t>Colonne1</t>
-        </is>
-      </c>
-      <c r="I56" s="11" t="inlineStr">
-        <is>
-          <t>Heures d’arrêt maladie</t>
-        </is>
-      </c>
-      <c r="J56" s="10" t="inlineStr">
-        <is>
-          <t>Heures de congés</t>
-        </is>
-      </c>
-      <c r="K56" s="10" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B57" s="61" t="n">
-        <v>46020</v>
-      </c>
-      <c r="C57" s="13" t="n">
-        <v>0.2916666666666667</v>
-      </c>
-      <c r="D57" s="13" t="n">
-        <v>0.5208333333333334</v>
-      </c>
-      <c r="E57" s="13" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="F57" s="13" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="G57" s="17">
-        <f>IFERROR(IF((((D57-C57)+(F57-E57))*24)&gt;8,8,((D57-C57)+(F57-E57))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H57" s="15" t="n"/>
-      <c r="I57" s="15" t="n"/>
-      <c r="J57" s="15" t="n"/>
-      <c r="K57" s="15" t="n"/>
-    </row>
-    <row r="58" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B58" s="61" t="n">
-        <v>46021</v>
-      </c>
-      <c r="C58" s="13" t="n"/>
-      <c r="D58" s="13" t="n"/>
-      <c r="E58" s="13" t="n"/>
-      <c r="F58" s="13" t="n"/>
-      <c r="G58" s="17">
-        <f>IFERROR(IF((((D58-C58)+(F58-E58))*24)&gt;8,8,((D58-C58)+(F58-E58))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H58" s="15" t="n"/>
-      <c r="I58" s="15" t="n"/>
-      <c r="J58" s="15" t="n"/>
-      <c r="K58" s="15">
-        <f>IFERROR(SUM(G58:J58), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B59" s="61" t="n">
-        <v>46022</v>
-      </c>
-      <c r="C59" s="13" t="n"/>
-      <c r="D59" s="13" t="n"/>
-      <c r="E59" s="13" t="n"/>
-      <c r="F59" s="13" t="n"/>
-      <c r="G59" s="17">
-        <f>IFERROR(IF((((D59-C59)+(F59-E59))*24)&gt;8,8,((D59-C59)+(F59-E59))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H59" s="15" t="n"/>
-      <c r="I59" s="15" t="n"/>
-      <c r="J59" s="15" t="n"/>
-      <c r="K59" s="15">
-        <f>IFERROR(SUM(G59:J59), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B60" s="61" t="n"/>
-      <c r="C60" s="13" t="n"/>
-      <c r="D60" s="13" t="n"/>
-      <c r="E60" s="13" t="n"/>
-      <c r="F60" s="13" t="n"/>
-      <c r="G60" s="17">
-        <f>IFERROR(IF((((D60-C60)+(F60-E60))*24)&gt;8,8,((D60-C60)+(F60-E60))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H60" s="15" t="n"/>
-      <c r="I60" s="15" t="n"/>
-      <c r="J60" s="15" t="n"/>
-      <c r="K60" s="15">
-        <f>IFERROR(SUM(G60:J60), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B61" s="61" t="n"/>
-      <c r="C61" s="13" t="n"/>
-      <c r="D61" s="13" t="n"/>
-      <c r="E61" s="13" t="n"/>
-      <c r="F61" s="13" t="n"/>
-      <c r="G61" s="17">
-        <f>IFERROR(IF((((D61-C61)+(F61-E61))*24)&gt;8,8,((D61-C61)+(F61-E61))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H61" s="15" t="n"/>
-      <c r="I61" s="15" t="n"/>
-      <c r="J61" s="15" t="n"/>
-      <c r="K61" s="15">
-        <f>IFERROR(SUM(G61:J61), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B62" s="61" t="n"/>
-      <c r="C62" s="13" t="n"/>
-      <c r="D62" s="13" t="n"/>
-      <c r="E62" s="13" t="n"/>
-      <c r="F62" s="13" t="n"/>
-      <c r="G62" s="17">
-        <f>IFERROR(IF((((D62-C62)+(F62-E62))*24)&gt;8,8,((D62-C62)+(F62-E62))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H62" s="15" t="n"/>
-      <c r="I62" s="15" t="n"/>
-      <c r="J62" s="15" t="n"/>
-      <c r="K62" s="15">
-        <f>IFERROR(SUM(G62:J62), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" hidden="1" ht="30" customHeight="1" s="58">
-      <c r="B63" s="61" t="n"/>
-      <c r="C63" s="13" t="n"/>
-      <c r="D63" s="13" t="n"/>
-      <c r="E63" s="13" t="n"/>
-      <c r="F63" s="13" t="n"/>
-      <c r="G63" s="17">
-        <f>IFERROR(IF((((D63-C63)+(F63-E63))*24)&gt;8,8,((D63-C63)+(F63-E63))*24), "")</f>
-        <v/>
-      </c>
-      <c r="H63" s="15" t="n"/>
-      <c r="I63" s="15" t="n"/>
-      <c r="J63" s="15" t="n"/>
-      <c r="K63" s="15">
-        <f>IFERROR(SUM(G63:J63), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" ht="30" customHeight="1" s="58">
-      <c r="F64" s="18" t="inlineStr">
-        <is>
-          <t>Nombre total d’heures</t>
-        </is>
-      </c>
-      <c r="G64" s="19">
-        <f>H19+H28+H37+H46</f>
-        <v/>
-      </c>
-      <c r="H64" s="19" t="n"/>
-      <c r="I64" s="19">
-        <f>SUM(I57:I63)</f>
-        <v/>
-      </c>
-      <c r="J64" s="19">
-        <f>SUM(J57:J63)</f>
-        <v/>
-      </c>
-      <c r="K64" s="21">
-        <f>SUM(TimeSheet367[Total])</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" ht="30" customHeight="1" s="58">
-      <c r="F65" s="22" t="inlineStr">
-        <is>
-          <t>Heures M-1</t>
-        </is>
-      </c>
-      <c r="G65" s="23" t="n">
-        <v>-3</v>
-      </c>
-      <c r="H65" s="62" t="n"/>
-      <c r="I65" s="62" t="n"/>
-      <c r="J65" s="62" t="n"/>
-      <c r="K65" s="63" t="n"/>
-    </row>
-    <row r="66" ht="30" customHeight="1" s="58">
-      <c r="F66" s="22" t="inlineStr">
-        <is>
-          <t>Reste heures</t>
-        </is>
-      </c>
-      <c r="G66" s="64">
-        <f>G65+G64</f>
-        <v/>
-      </c>
-      <c r="H66" s="65" t="n"/>
-      <c r="I66" s="65">
-        <f>I19*I65</f>
-        <v/>
-      </c>
-      <c r="J66" s="65">
-        <f>J19*J65</f>
-        <v/>
-      </c>
-      <c r="K66" s="65">
-        <f>SUM(G66:J66)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" ht="30" customHeight="1" s="58">
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-    </row>
+    <row r="20" ht="14.25" customHeight="1" s="58"/>
+    <row r="21" ht="30" customHeight="1" s="58"/>
+    <row r="22" ht="30" customHeight="1" s="58"/>
+    <row r="23" ht="30" customHeight="1" s="58"/>
+    <row r="24" ht="30" customHeight="1" s="58"/>
+    <row r="25" ht="30" customHeight="1" s="58"/>
+    <row r="26" ht="30" customHeight="1" s="58"/>
+    <row r="27" ht="30" customHeight="1" s="58"/>
+    <row r="28" ht="30" customHeight="1" s="58"/>
+    <row r="29" ht="14.25" customHeight="1" s="58"/>
+    <row r="30" ht="30" customHeight="1" s="58"/>
+    <row r="31" ht="30" customHeight="1" s="58"/>
+    <row r="32" ht="30" customHeight="1" s="58"/>
+    <row r="33" ht="30" customHeight="1" s="58"/>
+    <row r="34" ht="30" customHeight="1" s="58"/>
+    <row r="35" ht="30" customHeight="1" s="58"/>
+    <row r="36" ht="30" customHeight="1" s="58"/>
+    <row r="37" ht="30" customHeight="1" s="58"/>
+    <row r="38" ht="14.25" customHeight="1" s="58"/>
+    <row r="39" ht="30" customHeight="1" s="58"/>
+    <row r="40" ht="30" customHeight="1" s="58"/>
+    <row r="41" ht="30" customHeight="1" s="58"/>
+    <row r="42" ht="30" customHeight="1" s="58"/>
+    <row r="43" ht="30" customHeight="1" s="58"/>
+    <row r="44" ht="30" customHeight="1" s="58"/>
+    <row r="45" ht="30" customHeight="1" s="58"/>
+    <row r="46" ht="30" customHeight="1" s="58"/>
+    <row r="47" hidden="1" ht="14.25" customHeight="1" s="58"/>
+    <row r="48" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="49" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="50" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="51" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="52" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="53" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="54" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="55" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="56" hidden="1" ht="14.25" customHeight="1" s="58"/>
+    <row r="57" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="58" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="59" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="60" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="61" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="62" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="63" hidden="1" ht="30" customHeight="1" s="58"/>
+    <row r="64" ht="30" customHeight="1" s="58"/>
+    <row r="65" ht="30" customHeight="1" s="58"/>
+    <row r="66" ht="30" customHeight="1" s="58"/>
+    <row r="73" ht="30" customHeight="1" s="58"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="C6:H6"/>

</xml_diff>

<commit_message>
feat(rh): période de paie libre du→au + fonds de cellules du modèle
Exports paie / Silae / feuilles de temps sur plage libre (?du&au,
ex. 26/07 → 25/08), le mois restant la valeur par défaut. La fin du
dernier export paie est mémorisée (maquignon.heures_export_fin, par
société) et préremplit « du » = lendemain, « au » = aujourd'hui dans
le tableau des heures ; la plage s'applique aux 3 exports et aux 📄.

Fonds de cellules : le modèle utilise un tableau Excel structuré au
style personnalisé « Feuille de temps hebdomadaire » que copy_worksheet
ne recopie pas — tableau recréé sur chaque feuille (nom unique TS_Sxx,
formule =SUM(TS_Sxx[Total]) ajustée), 5 tableaux orphelins purgés du
gabarit.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XA7hsDjgUhFae2VXUBXjih
</commit_message>
<xml_diff>
--- a/feuille_temps_template.xlsx
+++ b/feuille_temps_template.xlsx
@@ -14695,127 +14695,6 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TimeSheet3" displayName="TimeSheet3" ref="B20:K27" headerRowCount="1" headerRowDxfId="894" dataDxfId="893" totalsRowDxfId="892">
-  <autoFilter ref="B20:K27"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="Jour" totalsRowLabel="Total" dataDxfId="891"/>
-    <tableColumn id="2" name="Arrivée" dataDxfId="890" totalsRowDxfId="889" dataCellStyle="Heure"/>
-    <tableColumn id="3" name="Départ" dataDxfId="888" totalsRowDxfId="887" dataCellStyle="Heure"/>
-    <tableColumn id="4" name="Arrivée " dataDxfId="886" totalsRowDxfId="885" dataCellStyle="Heure"/>
-    <tableColumn id="5" name="Départ " dataDxfId="884" totalsRowDxfId="883" dataCellStyle="Heure"/>
-    <tableColumn id="6" name="Heures normales" dataDxfId="882" totalsRowDxfId="881" dataCellStyle="Heures">
-      <calculatedColumnFormula>(D21-C21)+(F21-E21)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="7" name="Heures supplémentaires" dataDxfId="880" totalsRowDxfId="879" dataCellStyle="Heures">
-      <calculatedColumnFormula>ABS((G21-E1)*24)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="8" name="Heures d’arrêt maladie" dataDxfId="878" totalsRowDxfId="877" dataCellStyle="Heures"/>
-    <tableColumn id="9" name="Heures de congés" dataDxfId="876" totalsRowDxfId="875" dataCellStyle="Heures"/>
-    <tableColumn id="10" name="Total" totalsRowFunction="sum" dataDxfId="874" totalsRowDxfId="873" dataCellStyle="Heures">
-      <calculatedColumnFormula>IFERROR(SUM(G21:J21), "")</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Feuille de temps hebdomadaire" showFirstColumn="1" showLastColumn="1" showRowStripes="0" showColumnStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TimeSheet34" displayName="TimeSheet34" ref="B29:K36" headerRowCount="1" headerRowDxfId="872" dataDxfId="871" totalsRowDxfId="870">
-  <autoFilter ref="B29:K36"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="Jour" totalsRowLabel="Total" dataDxfId="869"/>
-    <tableColumn id="2" name="Arrivée" dataDxfId="868" totalsRowDxfId="867" dataCellStyle="Heure"/>
-    <tableColumn id="3" name="Départ" dataDxfId="866" totalsRowDxfId="865" dataCellStyle="Heure"/>
-    <tableColumn id="4" name="Arrivée " dataDxfId="864" totalsRowDxfId="863" dataCellStyle="Heure"/>
-    <tableColumn id="5" name="Départ " dataDxfId="862" totalsRowDxfId="861" dataCellStyle="Heure"/>
-    <tableColumn id="6" name="Heures normales" dataDxfId="860" totalsRowDxfId="859" dataCellStyle="Heures">
-      <calculatedColumnFormula>(D30-C30)+(F30-E30)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="7" name="Heures supplémentaires" dataDxfId="858" dataCellStyle="Heures">
-      <calculatedColumnFormula>IFERROR(IF(((D30-C30)+(F30-E30))*24&gt;8,((D30-C30)+(F30-E30))*24-8,0), "")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="8" name="Heures d’arrêt maladie" dataDxfId="857" totalsRowDxfId="856" dataCellStyle="Heures"/>
-    <tableColumn id="9" name="Heures de congés" dataDxfId="855" totalsRowDxfId="854" dataCellStyle="Heures"/>
-    <tableColumn id="10" name="Total" totalsRowFunction="sum" dataDxfId="853" totalsRowDxfId="852" dataCellStyle="Heures">
-      <calculatedColumnFormula>IFERROR(SUM(G30:J30), "")</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Feuille de temps hebdomadaire" showFirstColumn="1" showLastColumn="1" showRowStripes="0" showColumnStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TimeSheet35" displayName="TimeSheet35" ref="B38:K45" headerRowCount="1" headerRowDxfId="851" dataDxfId="850" totalsRowDxfId="849">
-  <autoFilter ref="B38:K45"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="Jour" totalsRowLabel="Total" dataDxfId="848"/>
-    <tableColumn id="2" name="Arrivée" dataDxfId="847" totalsRowDxfId="846" dataCellStyle="Heure"/>
-    <tableColumn id="3" name="Départ" dataDxfId="845" totalsRowDxfId="844" dataCellStyle="Heure"/>
-    <tableColumn id="4" name="Arrivée " dataDxfId="843" totalsRowDxfId="842" dataCellStyle="Heure"/>
-    <tableColumn id="5" name="Départ " dataDxfId="841" totalsRowDxfId="840" dataCellStyle="Heure"/>
-    <tableColumn id="6" name="Heures normales" dataDxfId="839" totalsRowDxfId="838" dataCellStyle="Heures">
-      <calculatedColumnFormula>(D39-C39)+(F39-E39)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="7" name="Heures supplémentaires" dataDxfId="837" totalsRowDxfId="836" dataCellStyle="Heures">
-      <calculatedColumnFormula>(G39-E1)*24</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="8" name="Heures d’arrêt maladie" dataDxfId="835" totalsRowDxfId="834" dataCellStyle="Heures"/>
-    <tableColumn id="9" name="Heures de congés" dataDxfId="833" totalsRowDxfId="832" dataCellStyle="Heures"/>
-    <tableColumn id="10" name="Total" totalsRowFunction="sum" dataDxfId="831" totalsRowDxfId="830" dataCellStyle="Heures">
-      <calculatedColumnFormula>IFERROR(SUM(G39:J39), "")</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Feuille de temps hebdomadaire" showFirstColumn="1" showLastColumn="1" showRowStripes="0" showColumnStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TimeSheet36" displayName="TimeSheet36" ref="B47:K54" headerRowCount="1" headerRowDxfId="829" dataDxfId="828" totalsRowDxfId="827">
-  <autoFilter ref="B47:K54"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="Jour" totalsRowLabel="Total" dataDxfId="826"/>
-    <tableColumn id="2" name="Arrivée" dataDxfId="825" totalsRowDxfId="824" dataCellStyle="Heure"/>
-    <tableColumn id="3" name="Départ" dataDxfId="823" totalsRowDxfId="822" dataCellStyle="Heure"/>
-    <tableColumn id="4" name="Arrivée " dataDxfId="821" totalsRowDxfId="820" dataCellStyle="Heure"/>
-    <tableColumn id="5" name="Départ " dataDxfId="819" totalsRowDxfId="818" dataCellStyle="Heure"/>
-    <tableColumn id="6" name="Heures normales" dataDxfId="817" totalsRowDxfId="816" dataCellStyle="Heures">
-      <calculatedColumnFormula>IFERROR(IF((((D48-C48)+(F48-E48))*24)&gt;8,8,((D48-C48)+(F48-E48))*24), "")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="7" name="Colonne1" dataDxfId="815" totalsRowDxfId="814" dataCellStyle="Heures"/>
-    <tableColumn id="8" name="Heures d’arrêt maladie" dataDxfId="813" totalsRowDxfId="812" dataCellStyle="Heures"/>
-    <tableColumn id="9" name="Heures de congés" dataDxfId="811" totalsRowDxfId="810" dataCellStyle="Heures"/>
-    <tableColumn id="10" name="Total" totalsRowFunction="sum" dataDxfId="809" totalsRowDxfId="808" dataCellStyle="Heures">
-      <calculatedColumnFormula>IFERROR(SUM(G48:J48), "")</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Feuille de temps hebdomadaire" showFirstColumn="1" showLastColumn="1" showRowStripes="0" showColumnStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TimeSheet367" displayName="TimeSheet367" ref="B56:K63" headerRowCount="1" headerRowDxfId="807" dataDxfId="806" totalsRowDxfId="805">
-  <autoFilter ref="B56:K63"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="Jour" totalsRowLabel="Total" dataDxfId="804"/>
-    <tableColumn id="2" name="Arrivée" dataDxfId="803" totalsRowDxfId="802" dataCellStyle="Heure"/>
-    <tableColumn id="3" name="Départ" dataDxfId="801" totalsRowDxfId="800" dataCellStyle="Heure"/>
-    <tableColumn id="4" name="Arrivée " dataDxfId="799" totalsRowDxfId="798" dataCellStyle="Heure"/>
-    <tableColumn id="5" name="Départ " dataDxfId="797" totalsRowDxfId="796" dataCellStyle="Heure"/>
-    <tableColumn id="6" name="Heures normales" dataDxfId="795" totalsRowDxfId="794" dataCellStyle="Heures">
-      <calculatedColumnFormula>IFERROR(IF((((D57-C57)+(F57-E57))*24)&gt;8,8,((D57-C57)+(F57-E57))*24), "")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="7" name="Colonne1" dataDxfId="793" totalsRowDxfId="792" dataCellStyle="Heures"/>
-    <tableColumn id="8" name="Heures d’arrêt maladie" dataDxfId="791" totalsRowDxfId="790" dataCellStyle="Heures"/>
-    <tableColumn id="9" name="Heures de congés" dataDxfId="789" totalsRowDxfId="788" dataCellStyle="Heures"/>
-    <tableColumn id="10" name="Total" totalsRowFunction="sum" dataDxfId="787" totalsRowDxfId="786" dataCellStyle="Heures">
-      <calculatedColumnFormula>IFERROR(SUM(G57:J57), "")</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Feuille de temps hebdomadaire" showFirstColumn="1" showLastColumn="1" showRowStripes="0" showColumnStripes="1"/>
-</table>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -15246,7 +15125,11 @@
           <t>Adresse e-mail de l’employé :</t>
         </is>
       </c>
-      <c r="K8" s="55" t="n"/>
+      <c r="K8" s="55" t="inlineStr">
+        <is>
+          <t>mailto:miguel@firstupconsultants.com</t>
+        </is>
+      </c>
     </row>
     <row r="9" hidden="1" ht="30" customHeight="1" s="58">
       <c r="B9" s="5" t="inlineStr">
@@ -15254,7 +15137,11 @@
           <t>E-mail :</t>
         </is>
       </c>
-      <c r="C9" s="55" t="n"/>
+      <c r="C9" s="55" t="inlineStr">
+        <is>
+          <t>mailto:first@firstupconsultants.com</t>
+        </is>
+      </c>
       <c r="D9" s="59" t="n"/>
       <c r="E9" s="59" t="n"/>
       <c r="F9" s="59" t="n"/>
@@ -15556,13 +15443,8 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <tableParts count="6">
+  <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>